<commit_message>
code working for garments, needs to improve model performance
</commit_message>
<xml_diff>
--- a/Data/Sheet.xlsx
+++ b/Data/Sheet.xlsx
@@ -445,7 +445,7 @@
         <v>Full Color</v>
       </c>
       <c r="F2" t="str">
-        <v>Full Back</v>
+        <v>Left Hip Right Hip</v>
       </c>
       <c r="G2" t="str">
         <v>240MFSilver-9904775_7811730.jpg</v>
@@ -454,7 +454,7 @@
         <v>Welspun</v>
       </c>
       <c r="I2" t="str">
-        <v>1. FULL-BACK</v>
+        <v>1. LEFT-HIP-RIGHT-HIP</v>
       </c>
     </row>
     <row r="3">

</xml_diff>